<commit_message>
Add exact method and submission writer; record S1/S2 exact results
- runner: --method exact (BlueQubit cpu device) writes values to Qubits!B
  ("Exact sample") and a Jobs row; config now targets the official IDs
  Duke_<C>_<q> for S1-S3 and G1-G4, plus a demo circuit for offline tests
- scripts/write_submission.py: per-circuit CSV (circuit_id,value) saved as
  submissions/<circuit>_v<N>.csv, with the upload page's checks
- S1 (4 qubits) and S2 (16 qubits) computed exactly at 0 credits; values match
  a local statevector simulation of the sample QASM files to within 2e-7

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/runs/sample_1.xlsx
+++ b/runs/sample_1.xlsx
@@ -7,6 +7,7 @@
     <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Estimates" sheetId="3" r:id="R1d720d84aca54612"/>
     <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Jobs" sheetId="4" r:id="R6973999336ec48c7"/>
   </x:sheets>
+  <x:calcPr fullCalcOnLoad="1"/>
 </x:workbook>
 </file>
 
@@ -464,7 +465,11 @@
       <x:c r="A4" s="2" t="str">
         <x:v>Official circuit ID</x:v>
       </x:c>
-      <x:c r="B4" s="6"/>
+      <x:c r="B4" s="6" t="inlineStr">
+        <x:is>
+          <x:t>S1</x:t>
+        </x:is>
+      </x:c>
       <x:c r="C4" s="2"/>
       <x:c r="D4" s="11" t="str">
         <x:v>Precision settings</x:v>
@@ -484,7 +489,9 @@
       <x:c r="A5" s="2" t="str">
         <x:v>Required qubits</x:v>
       </x:c>
-      <x:c r="B5" s="6"/>
+      <x:c r="B5" s="6" t="n">
+        <x:v>4</x:v>
+      </x:c>
       <x:c r="C5" s="2"/>
       <x:c r="D5" s="2" t="str">
         <x:v>MPS bond dimension χ</x:v>
@@ -1158,8 +1165,12 @@
       </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="20"/>
-      <x:c r="B6" s="19"/>
+      <x:c r="A6" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="B6" s="19" t="n">
+        <x:v>-0.3621922593901457</x:v>
+      </x:c>
       <x:c r="C6" s="14" t="str">
         <x:f>IF(OR(COUNTA($A6)=0,NOT(ISNUMBER('Status'!$E$5))),"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A6,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)=0,"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A6,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)&gt;1,"DUP",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A6,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1,'Estimates'!$F$5:$F$2004,"&lt;&gt;")=0,"",SUMIFS('Estimates'!$F$5:$F$2004,'Estimates'!$A$5:$A$2004,$A6,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)))))</x:f>
       </x:c>
@@ -1214,8 +1225,12 @@
       </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="20"/>
-      <x:c r="B7" s="19"/>
+      <x:c r="A7" s="20" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B7" s="19" t="n">
+        <x:v>-0.23266735629776267</x:v>
+      </x:c>
       <x:c r="C7" s="14" t="str">
         <x:f>IF(OR(COUNTA($A7)=0,NOT(ISNUMBER('Status'!$E$5))),"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A7,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)=0,"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A7,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)&gt;1,"DUP",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A7,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1,'Estimates'!$F$5:$F$2004,"&lt;&gt;")=0,"",SUMIFS('Estimates'!$F$5:$F$2004,'Estimates'!$A$5:$A$2004,$A7,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)))))</x:f>
       </x:c>
@@ -1270,8 +1285,12 @@
       </x:c>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="20"/>
-      <x:c r="B8" s="19"/>
+      <x:c r="A8" s="20" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B8" s="19" t="n">
+        <x:v>0.10250411538796315</x:v>
+      </x:c>
       <x:c r="C8" s="14" t="str">
         <x:f>IF(OR(COUNTA($A8)=0,NOT(ISNUMBER('Status'!$E$5))),"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A8,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)=0,"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A8,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)&gt;1,"DUP",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A8,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1,'Estimates'!$F$5:$F$2004,"&lt;&gt;")=0,"",SUMIFS('Estimates'!$F$5:$F$2004,'Estimates'!$A$5:$A$2004,$A8,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)))))</x:f>
       </x:c>
@@ -1326,8 +1345,12 @@
       </x:c>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="20"/>
-      <x:c r="B9" s="19"/>
+      <x:c r="A9" s="20" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B9" s="19" t="n">
+        <x:v>-0.10937094850563352</x:v>
+      </x:c>
       <x:c r="C9" s="14" t="str">
         <x:f>IF(OR(COUNTA($A9)=0,NOT(ISNUMBER('Status'!$E$5))),"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A9,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)=0,"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A9,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)&gt;1,"DUP",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A9,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1,'Estimates'!$F$5:$F$2004,"&lt;&gt;")=0,"",SUMIFS('Estimates'!$F$5:$F$2004,'Estimates'!$A$5:$A$2004,$A9,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)))))</x:f>
       </x:c>
@@ -18404,52 +18427,140 @@
       </x:c>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="6"/>
-      <x:c r="B5" s="6"/>
+      <x:c r="A5" s="6" t="inlineStr">
+        <x:is>
+          <x:t>bzMWdutLEuLfGnQS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B5" s="6" t="inlineStr">
+        <x:is>
+          <x:t>Exact</x:t>
+        </x:is>
+      </x:c>
       <x:c r="C5" s="6"/>
       <x:c r="D5" s="12"/>
       <x:c r="E5" s="6"/>
-      <x:c r="F5" s="6"/>
-      <x:c r="G5" s="6"/>
-      <x:c r="H5" s="8"/>
-      <x:c r="I5" s="8"/>
-      <x:c r="J5" s="6"/>
+      <x:c r="F5" s="6" t="inlineStr">
+        <x:is>
+          <x:t>succeeded</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G5" s="6" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H5" s="8" t="n">
+        <x:v>0.028</x:v>
+      </x:c>
+      <x:c r="I5" s="8" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J5" s="6" t="inlineStr">
+        <x:is>
+          <x:t>runner bb469474b4465930605b</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="6"/>
-      <x:c r="B6" s="6"/>
+      <x:c r="A6" s="6" t="inlineStr">
+        <x:is>
+          <x:t>vTlWoGMG8HxiH52f</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B6" s="6" t="inlineStr">
+        <x:is>
+          <x:t>Exact</x:t>
+        </x:is>
+      </x:c>
       <x:c r="C6" s="6"/>
       <x:c r="D6" s="12"/>
       <x:c r="E6" s="6"/>
-      <x:c r="F6" s="6"/>
-      <x:c r="G6" s="6"/>
-      <x:c r="H6" s="8"/>
-      <x:c r="I6" s="8"/>
-      <x:c r="J6" s="6"/>
+      <x:c r="F6" s="6" t="inlineStr">
+        <x:is>
+          <x:t>succeeded</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G6" s="6" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H6" s="8" t="n">
+        <x:v>0.026</x:v>
+      </x:c>
+      <x:c r="I6" s="8" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J6" s="6" t="inlineStr">
+        <x:is>
+          <x:t>runner 10c92b505fbedaf6373c</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="6"/>
-      <x:c r="B7" s="6"/>
+      <x:c r="A7" s="6" t="inlineStr">
+        <x:is>
+          <x:t>Ny0FhXGKFn1WFvJ0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B7" s="6" t="inlineStr">
+        <x:is>
+          <x:t>Exact</x:t>
+        </x:is>
+      </x:c>
       <x:c r="C7" s="6"/>
       <x:c r="D7" s="12"/>
       <x:c r="E7" s="6"/>
-      <x:c r="F7" s="6"/>
-      <x:c r="G7" s="6"/>
-      <x:c r="H7" s="8"/>
-      <x:c r="I7" s="8"/>
-      <x:c r="J7" s="6"/>
+      <x:c r="F7" s="6" t="inlineStr">
+        <x:is>
+          <x:t>succeeded</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G7" s="6" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H7" s="8" t="n">
+        <x:v>0.028</x:v>
+      </x:c>
+      <x:c r="I7" s="8" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J7" s="6" t="inlineStr">
+        <x:is>
+          <x:t>runner 332f7a15fd5250cc3086</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="6"/>
-      <x:c r="B8" s="6"/>
+      <x:c r="A8" s="6" t="inlineStr">
+        <x:is>
+          <x:t>gEJuPUHl9fnY1QIE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B8" s="6" t="inlineStr">
+        <x:is>
+          <x:t>Exact</x:t>
+        </x:is>
+      </x:c>
       <x:c r="C8" s="6"/>
       <x:c r="D8" s="12"/>
       <x:c r="E8" s="6"/>
-      <x:c r="F8" s="6"/>
-      <x:c r="G8" s="6"/>
-      <x:c r="H8" s="8"/>
-      <x:c r="I8" s="8"/>
-      <x:c r="J8" s="6"/>
+      <x:c r="F8" s="6" t="inlineStr">
+        <x:is>
+          <x:t>succeeded</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G8" s="6" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H8" s="8" t="n">
+        <x:v>0.027</x:v>
+      </x:c>
+      <x:c r="I8" s="8" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J8" s="6" t="inlineStr">
+        <x:is>
+          <x:t>runner 21cb152ac4c675dacf09</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="6"/>

</xml_diff>